<commit_message>
claude caude extension helped clean up model and the backtest. ready to run trials to find optimal stat mix
</commit_message>
<xml_diff>
--- a/predictions_log.xlsx
+++ b/predictions_log.xlsx
@@ -2843,11 +2843,15 @@
       <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="2" t="inlineStr"/>
       <c r="P32" s="2" t="inlineStr"/>
-      <c r="Q32" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="R32" s="2" t="n">
-        <v>2</v>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="S32" s="2" t="inlineStr">
         <is>
@@ -2906,11 +2910,15 @@
           <t>No Edge</t>
         </is>
       </c>
-      <c r="Q33" t="n">
-        <v>3</v>
-      </c>
-      <c r="R33" t="n">
-        <v>2</v>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
@@ -2977,11 +2985,15 @@
       <c r="N34" s="3" t="inlineStr"/>
       <c r="O34" s="3" t="inlineStr"/>
       <c r="P34" s="3" t="inlineStr"/>
-      <c r="Q34" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="R34" s="3" t="n">
-        <v>4</v>
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R34" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="S34" s="3" t="inlineStr">
         <is>
@@ -3040,11 +3052,15 @@
           <t>No Edge</t>
         </is>
       </c>
-      <c r="Q35" t="n">
-        <v>5</v>
-      </c>
-      <c r="R35" t="n">
-        <v>4</v>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
@@ -3111,11 +3127,15 @@
       <c r="N36" s="3" t="inlineStr"/>
       <c r="O36" s="3" t="inlineStr"/>
       <c r="P36" s="3" t="inlineStr"/>
-      <c r="Q36" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="R36" s="3" t="n">
-        <v>9</v>
+      <c r="Q36" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R36" s="3" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="S36" s="3" t="inlineStr">
         <is>
@@ -3174,11 +3194,15 @@
           <t>-2.5 runs</t>
         </is>
       </c>
-      <c r="Q37" t="n">
-        <v>1</v>
-      </c>
-      <c r="R37" t="n">
-        <v>9</v>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
@@ -3245,11 +3269,15 @@
       <c r="N38" s="2" t="inlineStr"/>
       <c r="O38" s="2" t="inlineStr"/>
       <c r="P38" s="2" t="inlineStr"/>
-      <c r="Q38" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="R38" s="2" t="n">
-        <v>2</v>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="S38" s="2" t="inlineStr">
         <is>
@@ -3308,11 +3336,15 @@
           <t>No Edge</t>
         </is>
       </c>
-      <c r="Q39" t="n">
-        <v>3</v>
-      </c>
-      <c r="R39" t="n">
-        <v>2</v>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
@@ -3379,11 +3411,15 @@
       <c r="N40" s="2" t="inlineStr"/>
       <c r="O40" s="2" t="inlineStr"/>
       <c r="P40" s="2" t="inlineStr"/>
-      <c r="Q40" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="R40" s="2" t="n">
-        <v>11</v>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="S40" s="2" t="inlineStr">
         <is>
@@ -3442,11 +3478,15 @@
           <t>No Edge</t>
         </is>
       </c>
-      <c r="Q41" t="n">
-        <v>9</v>
-      </c>
-      <c r="R41" t="n">
-        <v>11</v>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
@@ -3513,11 +3553,15 @@
       <c r="N42" s="3" t="inlineStr"/>
       <c r="O42" s="3" t="inlineStr"/>
       <c r="P42" s="3" t="inlineStr"/>
-      <c r="Q42" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="R42" s="3" t="n">
-        <v>2</v>
+      <c r="Q42" s="3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="R42" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="S42" s="3" t="inlineStr">
         <is>
@@ -3576,11 +3620,15 @@
           <t>No Edge</t>
         </is>
       </c>
-      <c r="Q43" t="n">
-        <v>7</v>
-      </c>
-      <c r="R43" t="n">
-        <v>2</v>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
@@ -3647,11 +3695,15 @@
       <c r="N44" s="2" t="inlineStr"/>
       <c r="O44" s="2" t="inlineStr"/>
       <c r="P44" s="2" t="inlineStr"/>
-      <c r="Q44" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="R44" s="2" t="n">
-        <v>7</v>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="S44" s="2" t="inlineStr">
         <is>
@@ -3710,11 +3762,15 @@
           <t>+2.0 runs</t>
         </is>
       </c>
-      <c r="Q45" t="n">
-        <v>6</v>
-      </c>
-      <c r="R45" t="n">
-        <v>7</v>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
@@ -3781,11 +3837,15 @@
       <c r="N46" s="2" t="inlineStr"/>
       <c r="O46" s="2" t="inlineStr"/>
       <c r="P46" s="2" t="inlineStr"/>
-      <c r="Q46" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="R46" s="2" t="n">
-        <v>10</v>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="S46" s="2" t="inlineStr">
         <is>
@@ -3844,11 +3904,15 @@
           <t>No Edge</t>
         </is>
       </c>
-      <c r="Q47" t="n">
-        <v>5</v>
-      </c>
-      <c r="R47" t="n">
-        <v>10</v>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
@@ -3915,11 +3979,15 @@
       <c r="N48" s="2" t="inlineStr"/>
       <c r="O48" s="2" t="inlineStr"/>
       <c r="P48" s="2" t="inlineStr"/>
-      <c r="Q48" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="R48" s="2" t="n">
-        <v>0</v>
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="S48" s="2" t="inlineStr">
         <is>
@@ -3978,11 +4046,15 @@
           <t>No Edge</t>
         </is>
       </c>
-      <c r="Q49" t="n">
-        <v>2</v>
-      </c>
-      <c r="R49" t="n">
-        <v>0</v>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
@@ -4049,11 +4121,15 @@
       <c r="N50" s="3" t="inlineStr"/>
       <c r="O50" s="3" t="inlineStr"/>
       <c r="P50" s="3" t="inlineStr"/>
-      <c r="Q50" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="R50" s="3" t="n">
-        <v>3</v>
+      <c r="Q50" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R50" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="S50" s="3" t="inlineStr">
         <is>
@@ -4112,11 +4188,15 @@
           <t>No Edge</t>
         </is>
       </c>
-      <c r="Q51" t="n">
-        <v>2</v>
-      </c>
-      <c r="R51" t="n">
-        <v>3</v>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
@@ -4183,11 +4263,15 @@
       <c r="N52" s="3" t="inlineStr"/>
       <c r="O52" s="3" t="inlineStr"/>
       <c r="P52" s="3" t="inlineStr"/>
-      <c r="Q52" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="R52" s="3" t="n">
-        <v>2</v>
+      <c r="Q52" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R52" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="S52" s="3" t="inlineStr">
         <is>
@@ -4246,11 +4330,15 @@
           <t>No Edge</t>
         </is>
       </c>
-      <c r="Q53" t="n">
-        <v>3</v>
-      </c>
-      <c r="R53" t="n">
-        <v>2</v>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
@@ -4317,11 +4405,15 @@
       <c r="N54" s="2" t="inlineStr"/>
       <c r="O54" s="2" t="inlineStr"/>
       <c r="P54" s="2" t="inlineStr"/>
-      <c r="Q54" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="R54" s="2" t="n">
-        <v>5</v>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="S54" s="2" t="inlineStr">
         <is>
@@ -4380,11 +4472,15 @@
           <t>No Edge</t>
         </is>
       </c>
-      <c r="Q55" t="n">
-        <v>2</v>
-      </c>
-      <c r="R55" t="n">
-        <v>5</v>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
@@ -4451,11 +4547,15 @@
       <c r="N56" s="2" t="inlineStr"/>
       <c r="O56" s="2" t="inlineStr"/>
       <c r="P56" s="2" t="inlineStr"/>
-      <c r="Q56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R56" s="2" t="n">
-        <v>2</v>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R56" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="S56" s="2" t="inlineStr">
         <is>
@@ -4514,11 +4614,15 @@
           <t>No Edge</t>
         </is>
       </c>
-      <c r="Q57" t="n">
-        <v>0</v>
-      </c>
-      <c r="R57" t="n">
-        <v>2</v>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
@@ -4537,270 +4641,366 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
+      <c r="A58" s="1" t="inlineStr">
         <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B58" s="1" t="inlineStr">
         <is>
           <t>LAA</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C58" s="1" t="inlineStr">
         <is>
           <t>LAD</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
+      <c r="D58" s="1" t="inlineStr">
         <is>
           <t>Moneyline</t>
         </is>
       </c>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="E58" s="1" t="inlineStr">
         <is>
           <t>LAD</t>
         </is>
       </c>
-      <c r="F58" s="3" t="inlineStr">
+      <c r="F58" s="1" t="inlineStr">
         <is>
           <t>63.4%</t>
         </is>
       </c>
-      <c r="G58" s="3" t="inlineStr">
+      <c r="G58" s="1" t="inlineStr">
         <is>
           <t>-136</t>
         </is>
       </c>
-      <c r="H58" s="3" t="inlineStr">
+      <c r="H58" s="1" t="inlineStr">
         <is>
           <t>+5.8%</t>
         </is>
       </c>
-      <c r="I58" s="3" t="inlineStr"/>
-      <c r="J58" s="3" t="inlineStr"/>
-      <c r="K58" s="3" t="inlineStr"/>
-      <c r="L58" s="3" t="inlineStr"/>
-      <c r="M58" s="3" t="inlineStr"/>
-      <c r="N58" s="3" t="inlineStr"/>
-      <c r="O58" s="3" t="inlineStr"/>
-      <c r="P58" s="3" t="inlineStr"/>
-      <c r="Q58" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R58" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="S58" s="3" t="inlineStr">
+      <c r="I58" s="1" t="inlineStr"/>
+      <c r="J58" s="1" t="inlineStr"/>
+      <c r="K58" s="1" t="inlineStr"/>
+      <c r="L58" s="1" t="inlineStr"/>
+      <c r="M58" s="1" t="inlineStr">
         <is>
           <t>LAD</t>
         </is>
       </c>
-      <c r="T58" s="3" t="inlineStr">
+      <c r="N58" s="1" t="inlineStr">
+        <is>
+          <t>63.5%</t>
+        </is>
+      </c>
+      <c r="O58" s="1" t="inlineStr">
+        <is>
+          <t>-136</t>
+        </is>
+      </c>
+      <c r="P58" s="1" t="inlineStr">
+        <is>
+          <t>+5.8%</t>
+        </is>
+      </c>
+      <c r="Q58" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R58" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="S58" s="1" t="inlineStr">
+        <is>
+          <t>LAD</t>
+        </is>
+      </c>
+      <c r="T58" s="1" t="inlineStr">
         <is>
           <t>WIN</t>
         </is>
       </c>
-      <c r="U58" s="3" t="inlineStr">
-        <is>
-          <t>CONSISTENT</t>
+      <c r="U58" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="1" t="inlineStr">
         <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="1" t="inlineStr">
         <is>
           <t>LAA</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="1" t="inlineStr">
         <is>
           <t>LAD</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D59" s="1" t="inlineStr">
         <is>
           <t>Over/Under</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>No Bet</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
+      <c r="E59" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F59" s="1" t="inlineStr">
         <is>
           <t>7.2</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
+      <c r="G59" s="1" t="inlineStr">
         <is>
           <t>8.5</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>No Edge</t>
-        </is>
-      </c>
-      <c r="Q59" t="n">
-        <v>0</v>
-      </c>
-      <c r="R59" t="n">
-        <v>6</v>
-      </c>
-      <c r="S59" t="inlineStr">
+      <c r="H59" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I59" s="1" t="inlineStr"/>
+      <c r="J59" s="1" t="inlineStr"/>
+      <c r="K59" s="1" t="inlineStr"/>
+      <c r="L59" s="1" t="inlineStr"/>
+      <c r="M59" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N59" s="1" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="O59" s="1" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="P59" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q59" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R59" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="S59" s="1" t="inlineStr">
         <is>
           <t>LAD</t>
         </is>
       </c>
-      <c r="T59" t="inlineStr">
+      <c r="T59" s="1" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="U59" t="inlineStr">
-        <is>
-          <t>CONSISTENT</t>
+      <c r="U59" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+      <c r="A60" s="1" t="inlineStr">
         <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B60" s="1" t="inlineStr">
         <is>
           <t>ATH</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr">
+      <c r="C60" s="1" t="inlineStr">
         <is>
           <t>SFG</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="D60" s="1" t="inlineStr">
         <is>
           <t>Moneyline</t>
         </is>
       </c>
-      <c r="E60" s="3" t="inlineStr">
+      <c r="E60" s="1" t="inlineStr">
         <is>
           <t>ATH</t>
         </is>
       </c>
-      <c r="F60" s="3" t="inlineStr">
+      <c r="F60" s="1" t="inlineStr">
         <is>
           <t>68.8%</t>
         </is>
       </c>
-      <c r="G60" s="3" t="inlineStr">
+      <c r="G60" s="1" t="inlineStr">
         <is>
           <t>-134</t>
         </is>
       </c>
-      <c r="H60" s="3" t="inlineStr">
+      <c r="H60" s="1" t="inlineStr">
         <is>
           <t>+11.5%</t>
         </is>
       </c>
-      <c r="I60" s="3" t="inlineStr"/>
-      <c r="J60" s="3" t="inlineStr"/>
-      <c r="K60" s="3" t="inlineStr"/>
-      <c r="L60" s="3" t="inlineStr"/>
-      <c r="M60" s="3" t="inlineStr"/>
-      <c r="N60" s="3" t="inlineStr"/>
-      <c r="O60" s="3" t="inlineStr"/>
-      <c r="P60" s="3" t="inlineStr"/>
-      <c r="Q60" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="R60" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="S60" s="3" t="inlineStr">
+      <c r="I60" s="1" t="inlineStr"/>
+      <c r="J60" s="1" t="inlineStr"/>
+      <c r="K60" s="1" t="inlineStr"/>
+      <c r="L60" s="1" t="inlineStr"/>
+      <c r="M60" s="1" t="inlineStr">
         <is>
           <t>ATH</t>
         </is>
       </c>
-      <c r="T60" s="3" t="inlineStr">
+      <c r="N60" s="1" t="inlineStr">
+        <is>
+          <t>68.6%</t>
+        </is>
+      </c>
+      <c r="O60" s="1" t="inlineStr">
+        <is>
+          <t>-134</t>
+        </is>
+      </c>
+      <c r="P60" s="1" t="inlineStr">
+        <is>
+          <t>+11.4%</t>
+        </is>
+      </c>
+      <c r="Q60" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R60" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S60" s="1" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="T60" s="1" t="inlineStr">
         <is>
           <t>WIN</t>
         </is>
       </c>
-      <c r="U60" s="3" t="inlineStr">
-        <is>
-          <t>CONSISTENT</t>
+      <c r="U60" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="1" t="inlineStr">
         <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="1" t="inlineStr">
         <is>
           <t>ATH</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="1" t="inlineStr">
         <is>
           <t>SFG</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" s="1" t="inlineStr">
         <is>
           <t>Over/Under</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>No Bet</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
+      <c r="E61" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F61" s="1" t="inlineStr">
         <is>
           <t>9.2</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr">
+      <c r="G61" s="1" t="inlineStr">
         <is>
           <t>9.5</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>No Edge</t>
-        </is>
-      </c>
-      <c r="Q61" t="n">
-        <v>5</v>
-      </c>
-      <c r="R61" t="n">
-        <v>2</v>
-      </c>
-      <c r="S61" t="inlineStr">
+      <c r="H61" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I61" s="1" t="inlineStr"/>
+      <c r="J61" s="1" t="inlineStr"/>
+      <c r="K61" s="1" t="inlineStr"/>
+      <c r="L61" s="1" t="inlineStr"/>
+      <c r="M61" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N61" s="1" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="O61" s="1" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="P61" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q61" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R61" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S61" s="1" t="inlineStr">
         <is>
           <t>ATH</t>
         </is>
       </c>
-      <c r="T61" t="inlineStr">
+      <c r="T61" s="1" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="U61" t="inlineStr">
-        <is>
-          <t>CONSISTENT</t>
+      <c r="U61" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
backtest has been updated to run n times in a row - right now set for 3 - to speed up the trial runs
</commit_message>
<xml_diff>
--- a/predictions_log.xlsx
+++ b/predictions_log.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U61"/>
+  <dimension ref="A1:U85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5004,6 +5004,1790 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>TBR</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>TBR</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>64.6%</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>-148</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>+4.9%</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr"/>
+      <c r="M62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr"/>
+      <c r="O62" s="2" t="inlineStr"/>
+      <c r="P62" s="2" t="inlineStr"/>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R62" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="S62" s="2" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="T62" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U62" s="2" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>TBR</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>+2.3 runs</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>66.3%</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>-162</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>+4.5%</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr"/>
+      <c r="L64" s="2" t="inlineStr"/>
+      <c r="M64" s="2" t="inlineStr"/>
+      <c r="N64" s="2" t="inlineStr"/>
+      <c r="O64" s="2" t="inlineStr"/>
+      <c r="P64" s="2" t="inlineStr"/>
+      <c r="Q64" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R64" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S64" s="2" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="T64" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U64" s="2" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>WSN</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>BAL</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>WSN</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>66.3%</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>106</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>+17.8%</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="inlineStr"/>
+      <c r="J66" s="3" t="inlineStr"/>
+      <c r="K66" s="3" t="inlineStr"/>
+      <c r="L66" s="3" t="inlineStr"/>
+      <c r="M66" s="3" t="inlineStr"/>
+      <c r="N66" s="3" t="inlineStr"/>
+      <c r="O66" s="3" t="inlineStr"/>
+      <c r="P66" s="3" t="inlineStr"/>
+      <c r="Q66" s="3" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="R66" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S66" s="3" t="inlineStr">
+        <is>
+          <t>WSN</t>
+        </is>
+      </c>
+      <c r="T66" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="U66" s="3" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>WSN</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>BAL</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>WSN</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>61.0%</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>+13.4%</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="inlineStr"/>
+      <c r="J68" s="3" t="inlineStr"/>
+      <c r="K68" s="3" t="inlineStr"/>
+      <c r="L68" s="3" t="inlineStr"/>
+      <c r="M68" s="3" t="inlineStr"/>
+      <c r="N68" s="3" t="inlineStr"/>
+      <c r="O68" s="3" t="inlineStr"/>
+      <c r="P68" s="3" t="inlineStr"/>
+      <c r="Q68" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R68" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="S68" s="3" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="T68" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="U68" s="3" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>CLE</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>CIN</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>CLE</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>70.4%</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>-163</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>+8.4%</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="inlineStr"/>
+      <c r="J70" s="3" t="inlineStr"/>
+      <c r="K70" s="3" t="inlineStr"/>
+      <c r="L70" s="3" t="inlineStr"/>
+      <c r="M70" s="3" t="inlineStr"/>
+      <c r="N70" s="3" t="inlineStr"/>
+      <c r="O70" s="3" t="inlineStr"/>
+      <c r="P70" s="3" t="inlineStr"/>
+      <c r="Q70" s="3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="R70" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="S70" s="3" t="inlineStr">
+        <is>
+          <t>CLE</t>
+        </is>
+      </c>
+      <c r="T70" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="U70" s="3" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>CLE</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>CIN</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>+1.8 runs</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>CLE</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>66.3%</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>-126</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>+10.6%</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="inlineStr"/>
+      <c r="J72" s="3" t="inlineStr"/>
+      <c r="K72" s="3" t="inlineStr"/>
+      <c r="L72" s="3" t="inlineStr"/>
+      <c r="M72" s="3" t="inlineStr"/>
+      <c r="N72" s="3" t="inlineStr"/>
+      <c r="O72" s="3" t="inlineStr"/>
+      <c r="P72" s="3" t="inlineStr"/>
+      <c r="Q72" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R72" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S72" s="3" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="T72" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="U72" s="3" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>+2.0 runs</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>NYM</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>NYY</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>50.2%</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>-120</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr"/>
+      <c r="L74" s="2" t="inlineStr"/>
+      <c r="M74" s="2" t="inlineStr"/>
+      <c r="N74" s="2" t="inlineStr"/>
+      <c r="O74" s="2" t="inlineStr"/>
+      <c r="P74" s="2" t="inlineStr"/>
+      <c r="Q74" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="R74" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S74" s="2" t="inlineStr">
+        <is>
+          <t>NYM</t>
+        </is>
+      </c>
+      <c r="T74" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U74" s="2" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>NYM</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>NYY</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>7.7</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>NYM</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>CHW</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>CHC</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>CHW</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>53.5%</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>+6.8%</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="inlineStr"/>
+      <c r="J76" s="3" t="inlineStr"/>
+      <c r="K76" s="3" t="inlineStr"/>
+      <c r="L76" s="3" t="inlineStr"/>
+      <c r="M76" s="3" t="inlineStr"/>
+      <c r="N76" s="3" t="inlineStr"/>
+      <c r="O76" s="3" t="inlineStr"/>
+      <c r="P76" s="3" t="inlineStr"/>
+      <c r="Q76" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="R76" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S76" s="3" t="inlineStr">
+        <is>
+          <t>CHW</t>
+        </is>
+      </c>
+      <c r="T76" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="U76" s="3" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>CHW</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>CHC</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>CHW</t>
+        </is>
+      </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>HOU</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>51.3%</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>-118</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr"/>
+      <c r="L78" s="2" t="inlineStr"/>
+      <c r="M78" s="2" t="inlineStr"/>
+      <c r="N78" s="2" t="inlineStr"/>
+      <c r="O78" s="2" t="inlineStr"/>
+      <c r="P78" s="2" t="inlineStr"/>
+      <c r="Q78" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R78" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S78" s="2" t="inlineStr">
+        <is>
+          <t>HOU</t>
+        </is>
+      </c>
+      <c r="T78" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U78" s="2" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>HOU</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>HOU</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>KCR</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>51.3%</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>-114</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr"/>
+      <c r="K80" s="2" t="inlineStr"/>
+      <c r="L80" s="2" t="inlineStr"/>
+      <c r="M80" s="2" t="inlineStr"/>
+      <c r="N80" s="2" t="inlineStr"/>
+      <c r="O80" s="2" t="inlineStr"/>
+      <c r="P80" s="2" t="inlineStr"/>
+      <c r="Q80" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R80" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S80" s="2" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="T80" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U80" s="2" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>KCR</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>8.7</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B82" s="1" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="C82" s="1" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="D82" s="1" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E82" s="1" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="F82" s="1" t="inlineStr">
+        <is>
+          <t>77.6%</t>
+        </is>
+      </c>
+      <c r="G82" s="1" t="inlineStr">
+        <is>
+          <t>-144</t>
+        </is>
+      </c>
+      <c r="H82" s="1" t="inlineStr">
+        <is>
+          <t>+18.6%</t>
+        </is>
+      </c>
+      <c r="I82" s="1" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="J82" s="1" t="inlineStr">
+        <is>
+          <t>78.9%</t>
+        </is>
+      </c>
+      <c r="K82" s="1" t="inlineStr">
+        <is>
+          <t>-144</t>
+        </is>
+      </c>
+      <c r="L82" s="1" t="inlineStr">
+        <is>
+          <t>+19.9%</t>
+        </is>
+      </c>
+      <c r="M82" s="1" t="inlineStr"/>
+      <c r="N82" s="1" t="inlineStr"/>
+      <c r="O82" s="1" t="inlineStr"/>
+      <c r="P82" s="1" t="inlineStr"/>
+      <c r="Q82" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R82" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S82" s="1" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="T82" s="1" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U82" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B83" s="1" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="C83" s="1" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="D83" s="1" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E83" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F83" s="1" t="inlineStr">
+        <is>
+          <t>10.4</t>
+        </is>
+      </c>
+      <c r="G83" s="1" t="inlineStr">
+        <is>
+          <t>10.5</t>
+        </is>
+      </c>
+      <c r="H83" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I83" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="J83" s="1" t="inlineStr">
+        <is>
+          <t>10.5</t>
+        </is>
+      </c>
+      <c r="K83" s="1" t="inlineStr">
+        <is>
+          <t>10.5</t>
+        </is>
+      </c>
+      <c r="L83" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="M83" s="1" t="inlineStr"/>
+      <c r="N83" s="1" t="inlineStr"/>
+      <c r="O83" s="1" t="inlineStr"/>
+      <c r="P83" s="1" t="inlineStr"/>
+      <c r="Q83" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R83" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S83" s="1" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="T83" s="1" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U83" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B84" s="1" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="C84" s="1" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
+      </c>
+      <c r="D84" s="1" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E84" s="1" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="F84" s="1" t="inlineStr">
+        <is>
+          <t>68.4%</t>
+        </is>
+      </c>
+      <c r="G84" s="1" t="inlineStr">
+        <is>
+          <t>-148</t>
+        </is>
+      </c>
+      <c r="H84" s="1" t="inlineStr">
+        <is>
+          <t>+8.7%</t>
+        </is>
+      </c>
+      <c r="I84" s="1" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="J84" s="1" t="inlineStr">
+        <is>
+          <t>67.5%</t>
+        </is>
+      </c>
+      <c r="K84" s="1" t="inlineStr">
+        <is>
+          <t>-146</t>
+        </is>
+      </c>
+      <c r="L84" s="1" t="inlineStr">
+        <is>
+          <t>+8.2%</t>
+        </is>
+      </c>
+      <c r="M84" s="1" t="inlineStr"/>
+      <c r="N84" s="1" t="inlineStr"/>
+      <c r="O84" s="1" t="inlineStr"/>
+      <c r="P84" s="1" t="inlineStr"/>
+      <c r="Q84" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R84" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="S84" s="1" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
+      </c>
+      <c r="T84" s="1" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U84" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B85" s="1" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="C85" s="1" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
+      </c>
+      <c r="D85" s="1" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E85" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F85" s="1" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="G85" s="1" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="H85" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I85" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="J85" s="1" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="K85" s="1" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="L85" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="M85" s="1" t="inlineStr"/>
+      <c r="N85" s="1" t="inlineStr"/>
+      <c r="O85" s="1" t="inlineStr"/>
+      <c r="P85" s="1" t="inlineStr"/>
+      <c r="Q85" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R85" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="S85" s="1" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
+      </c>
+      <c r="T85" s="1" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U85" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated backtest with relief pitcher appearences by game from 2021-2025 from statcast. added relief pitcher fatigue and usage anaylsis to factor into edge computation. first 5 runs of 100 trials will occur. Afterwards the results of what generated the most ROI will be used to adjust the weights and anothe 5 runs of 100 trials will be run.
</commit_message>
<xml_diff>
--- a/predictions_log.xlsx
+++ b/predictions_log.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U85"/>
+  <dimension ref="A1:U103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6788,6 +6788,1044 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>69.5%</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>-148</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>+9.9%</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>LAA</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>69.7%</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>-129</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>+13.3%</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>LAA</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>54.9%</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>119</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>+9.3%</t>
+        </is>
+      </c>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>CHW</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>57.2%</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>-162</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>CHW</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>8.6</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>SDP</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>LAD</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>59.0%</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>-144</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>SDP</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>LAD</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>LAA</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr"/>
+      <c r="G96" s="2" t="inlineStr"/>
+      <c r="H96" s="2" t="inlineStr"/>
+      <c r="I96" s="2" t="inlineStr"/>
+      <c r="J96" s="2" t="inlineStr"/>
+      <c r="K96" s="2" t="inlineStr"/>
+      <c r="L96" s="2" t="inlineStr"/>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>60.2%</t>
+        </is>
+      </c>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>118</t>
+        </is>
+      </c>
+      <c r="P96" s="2" t="inlineStr">
+        <is>
+          <t>+14.3%</t>
+        </is>
+      </c>
+      <c r="Q96" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R96" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S96" s="2" t="inlineStr">
+        <is>
+          <t>LAA</t>
+        </is>
+      </c>
+      <c r="T96" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U96" s="2" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>LAA</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>9.8</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>LAA</t>
+        </is>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr"/>
+      <c r="G98" s="2" t="inlineStr"/>
+      <c r="H98" s="2" t="inlineStr"/>
+      <c r="I98" s="2" t="inlineStr"/>
+      <c r="J98" s="2" t="inlineStr"/>
+      <c r="K98" s="2" t="inlineStr"/>
+      <c r="L98" s="2" t="inlineStr"/>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>57.1%</t>
+        </is>
+      </c>
+      <c r="O98" s="2" t="inlineStr">
+        <is>
+          <t>-124</t>
+        </is>
+      </c>
+      <c r="P98" s="2" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q98" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="R98" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S98" s="2" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="T98" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U98" s="2" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>8.8</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>CHW</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr"/>
+      <c r="F100" s="2" t="inlineStr"/>
+      <c r="G100" s="2" t="inlineStr"/>
+      <c r="H100" s="2" t="inlineStr"/>
+      <c r="I100" s="2" t="inlineStr"/>
+      <c r="J100" s="2" t="inlineStr"/>
+      <c r="K100" s="2" t="inlineStr"/>
+      <c r="L100" s="2" t="inlineStr"/>
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
+          <t>62.7%</t>
+        </is>
+      </c>
+      <c r="O100" s="2" t="inlineStr">
+        <is>
+          <t>-149</t>
+        </is>
+      </c>
+      <c r="P100" s="2" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q100" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="R100" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S100" s="2" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="T100" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U100" s="2" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>CHW</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>SDP</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>LAD</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr"/>
+      <c r="F102" s="2" t="inlineStr"/>
+      <c r="G102" s="2" t="inlineStr"/>
+      <c r="H102" s="2" t="inlineStr"/>
+      <c r="I102" s="2" t="inlineStr"/>
+      <c r="J102" s="2" t="inlineStr"/>
+      <c r="K102" s="2" t="inlineStr"/>
+      <c r="L102" s="2" t="inlineStr"/>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
+          <t>58.8%</t>
+        </is>
+      </c>
+      <c r="O102" s="2" t="inlineStr">
+        <is>
+          <t>-156</t>
+        </is>
+      </c>
+      <c r="P102" s="2" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q102" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R102" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S102" s="2" t="inlineStr">
+        <is>
+          <t>SDP</t>
+        </is>
+      </c>
+      <c r="T102" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U102" s="2" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>SDP</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>LAD</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>6.8</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>SDP</t>
+        </is>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
final round of inital trials complete. tweaked weights and re ran the backtest. Further refinment being done.
</commit_message>
<xml_diff>
--- a/predictions_log.xlsx
+++ b/predictions_log.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U103"/>
+  <dimension ref="A1:U129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7826,6 +7826,2292 @@
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>CIN</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>57.9%</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>-144</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr"/>
+      <c r="J104" s="2" t="inlineStr"/>
+      <c r="K104" s="2" t="inlineStr"/>
+      <c r="L104" s="2" t="inlineStr"/>
+      <c r="M104" s="2" t="inlineStr"/>
+      <c r="N104" s="2" t="inlineStr"/>
+      <c r="O104" s="2" t="inlineStr"/>
+      <c r="P104" s="2" t="inlineStr"/>
+      <c r="Q104" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R104" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="S104" s="2" t="inlineStr">
+        <is>
+          <t>CIN</t>
+        </is>
+      </c>
+      <c r="T104" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U104" s="2" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>CIN</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>CIN</t>
+        </is>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>TBR</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>BAL</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>TBR</t>
+        </is>
+      </c>
+      <c r="F106" s="3" t="inlineStr">
+        <is>
+          <t>72.8%</t>
+        </is>
+      </c>
+      <c r="G106" s="3" t="inlineStr">
+        <is>
+          <t>-119</t>
+        </is>
+      </c>
+      <c r="H106" s="3" t="inlineStr">
+        <is>
+          <t>+18.4%</t>
+        </is>
+      </c>
+      <c r="I106" s="3" t="inlineStr"/>
+      <c r="J106" s="3" t="inlineStr"/>
+      <c r="K106" s="3" t="inlineStr"/>
+      <c r="L106" s="3" t="inlineStr"/>
+      <c r="M106" s="3" t="inlineStr"/>
+      <c r="N106" s="3" t="inlineStr"/>
+      <c r="O106" s="3" t="inlineStr"/>
+      <c r="P106" s="3" t="inlineStr"/>
+      <c r="Q106" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R106" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S106" s="3" t="inlineStr">
+        <is>
+          <t>TBR</t>
+        </is>
+      </c>
+      <c r="T106" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="U106" s="3" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>TBR</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>BAL</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>+1.7 runs</t>
+        </is>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>TBR</t>
+        </is>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>CONSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B108" s="1" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="C108" s="1" t="inlineStr">
+        <is>
+          <t>HOU</t>
+        </is>
+      </c>
+      <c r="D108" s="1" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E108" s="1" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="F108" s="1" t="inlineStr">
+        <is>
+          <t>62.7%</t>
+        </is>
+      </c>
+      <c r="G108" s="1" t="inlineStr">
+        <is>
+          <t>-146</t>
+        </is>
+      </c>
+      <c r="H108" s="1" t="inlineStr">
+        <is>
+          <t>+3.4%</t>
+        </is>
+      </c>
+      <c r="I108" s="1" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="J108" s="1" t="inlineStr">
+        <is>
+          <t>62.7%</t>
+        </is>
+      </c>
+      <c r="K108" s="1" t="inlineStr">
+        <is>
+          <t>-142</t>
+        </is>
+      </c>
+      <c r="L108" s="1" t="inlineStr">
+        <is>
+          <t>+4.0%</t>
+        </is>
+      </c>
+      <c r="M108" s="1" t="inlineStr"/>
+      <c r="N108" s="1" t="inlineStr"/>
+      <c r="O108" s="1" t="inlineStr"/>
+      <c r="P108" s="1" t="inlineStr"/>
+      <c r="Q108" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R108" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S108" s="1" t="inlineStr">
+        <is>
+          <t>HOU</t>
+        </is>
+      </c>
+      <c r="T108" s="1" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U108" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B109" s="1" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="C109" s="1" t="inlineStr">
+        <is>
+          <t>HOU</t>
+        </is>
+      </c>
+      <c r="D109" s="1" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E109" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F109" s="1" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="G109" s="1" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="H109" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I109" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="J109" s="1" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="K109" s="1" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="L109" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="M109" s="1" t="inlineStr"/>
+      <c r="N109" s="1" t="inlineStr"/>
+      <c r="O109" s="1" t="inlineStr"/>
+      <c r="P109" s="1" t="inlineStr"/>
+      <c r="Q109" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R109" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S109" s="1" t="inlineStr">
+        <is>
+          <t>HOU</t>
+        </is>
+      </c>
+      <c r="T109" s="1" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U109" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B110" s="1" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="C110" s="1" t="inlineStr">
+        <is>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="D110" s="1" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E110" s="1" t="inlineStr">
+        <is>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="F110" s="1" t="inlineStr">
+        <is>
+          <t>78.0%</t>
+        </is>
+      </c>
+      <c r="G110" s="1" t="inlineStr">
+        <is>
+          <t>-126</t>
+        </is>
+      </c>
+      <c r="H110" s="1" t="inlineStr">
+        <is>
+          <t>+22.2%</t>
+        </is>
+      </c>
+      <c r="I110" s="1" t="inlineStr">
+        <is>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="J110" s="1" t="inlineStr">
+        <is>
+          <t>78.6%</t>
+        </is>
+      </c>
+      <c r="K110" s="1" t="inlineStr">
+        <is>
+          <t>-118</t>
+        </is>
+      </c>
+      <c r="L110" s="1" t="inlineStr">
+        <is>
+          <t>+24.5%</t>
+        </is>
+      </c>
+      <c r="M110" s="1" t="inlineStr"/>
+      <c r="N110" s="1" t="inlineStr"/>
+      <c r="O110" s="1" t="inlineStr"/>
+      <c r="P110" s="1" t="inlineStr"/>
+      <c r="Q110" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R110" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="S110" s="1" t="inlineStr">
+        <is>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="T110" s="1" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="U110" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B111" s="1" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="C111" s="1" t="inlineStr">
+        <is>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="D111" s="1" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E111" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F111" s="1" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="G111" s="1" t="inlineStr">
+        <is>
+          <t>10.5</t>
+        </is>
+      </c>
+      <c r="H111" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I111" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="J111" s="1" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="K111" s="1" t="inlineStr">
+        <is>
+          <t>10.5</t>
+        </is>
+      </c>
+      <c r="L111" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="M111" s="1" t="inlineStr"/>
+      <c r="N111" s="1" t="inlineStr"/>
+      <c r="O111" s="1" t="inlineStr"/>
+      <c r="P111" s="1" t="inlineStr"/>
+      <c r="Q111" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R111" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="S111" s="1" t="inlineStr">
+        <is>
+          <t>TEX</t>
+        </is>
+      </c>
+      <c r="T111" s="1" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U111" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B112" s="1" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="C112" s="1" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
+      </c>
+      <c r="D112" s="1" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E112" s="1" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="F112" s="1" t="inlineStr">
+        <is>
+          <t>66.0%</t>
+        </is>
+      </c>
+      <c r="G112" s="1" t="inlineStr">
+        <is>
+          <t>-130</t>
+        </is>
+      </c>
+      <c r="H112" s="1" t="inlineStr">
+        <is>
+          <t>+9.5%</t>
+        </is>
+      </c>
+      <c r="I112" s="1" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="J112" s="1" t="inlineStr">
+        <is>
+          <t>66.8%</t>
+        </is>
+      </c>
+      <c r="K112" s="1" t="inlineStr">
+        <is>
+          <t>-132</t>
+        </is>
+      </c>
+      <c r="L112" s="1" t="inlineStr">
+        <is>
+          <t>+9.9%</t>
+        </is>
+      </c>
+      <c r="M112" s="1" t="inlineStr"/>
+      <c r="N112" s="1" t="inlineStr"/>
+      <c r="O112" s="1" t="inlineStr"/>
+      <c r="P112" s="1" t="inlineStr"/>
+      <c r="Q112" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R112" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S112" s="1" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="T112" s="1" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="U112" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B113" s="1" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="C113" s="1" t="inlineStr">
+        <is>
+          <t>SFG</t>
+        </is>
+      </c>
+      <c r="D113" s="1" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E113" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F113" s="1" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="G113" s="1" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="H113" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I113" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="J113" s="1" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="K113" s="1" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="L113" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="M113" s="1" t="inlineStr"/>
+      <c r="N113" s="1" t="inlineStr"/>
+      <c r="O113" s="1" t="inlineStr"/>
+      <c r="P113" s="1" t="inlineStr"/>
+      <c r="Q113" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R113" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S113" s="1" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="T113" s="1" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U113" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B114" s="1" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="C114" s="1" t="inlineStr">
+        <is>
+          <t>CHW</t>
+        </is>
+      </c>
+      <c r="D114" s="1" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E114" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F114" s="1" t="inlineStr">
+        <is>
+          <t>62.6%</t>
+        </is>
+      </c>
+      <c r="G114" s="1" t="inlineStr">
+        <is>
+          <t>-154</t>
+        </is>
+      </c>
+      <c r="H114" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I114" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="J114" s="1" t="inlineStr">
+        <is>
+          <t>61.8%</t>
+        </is>
+      </c>
+      <c r="K114" s="1" t="inlineStr">
+        <is>
+          <t>-144</t>
+        </is>
+      </c>
+      <c r="L114" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="M114" s="1" t="inlineStr"/>
+      <c r="N114" s="1" t="inlineStr"/>
+      <c r="O114" s="1" t="inlineStr"/>
+      <c r="P114" s="1" t="inlineStr"/>
+      <c r="Q114" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R114" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S114" s="1" t="inlineStr">
+        <is>
+          <t>CHW</t>
+        </is>
+      </c>
+      <c r="T114" s="1" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U114" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B115" s="1" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="C115" s="1" t="inlineStr">
+        <is>
+          <t>CHW</t>
+        </is>
+      </c>
+      <c r="D115" s="1" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E115" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F115" s="1" t="inlineStr">
+        <is>
+          <t>7.7</t>
+        </is>
+      </c>
+      <c r="G115" s="1" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="H115" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I115" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="J115" s="1" t="inlineStr">
+        <is>
+          <t>7.6</t>
+        </is>
+      </c>
+      <c r="K115" s="1" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="L115" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="M115" s="1" t="inlineStr"/>
+      <c r="N115" s="1" t="inlineStr"/>
+      <c r="O115" s="1" t="inlineStr"/>
+      <c r="P115" s="1" t="inlineStr"/>
+      <c r="Q115" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R115" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S115" s="1" t="inlineStr">
+        <is>
+          <t>CHW</t>
+        </is>
+      </c>
+      <c r="T115" s="1" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U115" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B116" s="1" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="C116" s="1" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="D116" s="1" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E116" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F116" s="1" t="inlineStr">
+        <is>
+          <t>67.0%</t>
+        </is>
+      </c>
+      <c r="G116" s="1" t="inlineStr">
+        <is>
+          <t>-194</t>
+        </is>
+      </c>
+      <c r="H116" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I116" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="J116" s="1" t="inlineStr">
+        <is>
+          <t>67.2%</t>
+        </is>
+      </c>
+      <c r="K116" s="1" t="inlineStr">
+        <is>
+          <t>-188</t>
+        </is>
+      </c>
+      <c r="L116" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="M116" s="1" t="inlineStr"/>
+      <c r="N116" s="1" t="inlineStr"/>
+      <c r="O116" s="1" t="inlineStr"/>
+      <c r="P116" s="1" t="inlineStr"/>
+      <c r="Q116" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R116" s="1" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="S116" s="1" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="T116" s="1" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U116" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B117" s="1" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="C117" s="1" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="D117" s="1" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E117" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F117" s="1" t="inlineStr">
+        <is>
+          <t>7.7</t>
+        </is>
+      </c>
+      <c r="G117" s="1" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="H117" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I117" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="J117" s="1" t="inlineStr">
+        <is>
+          <t>7.7</t>
+        </is>
+      </c>
+      <c r="K117" s="1" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="L117" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="M117" s="1" t="inlineStr"/>
+      <c r="N117" s="1" t="inlineStr"/>
+      <c r="O117" s="1" t="inlineStr"/>
+      <c r="P117" s="1" t="inlineStr"/>
+      <c r="Q117" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R117" s="1" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="S117" s="1" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="T117" s="1" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U117" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B118" s="1" t="inlineStr">
+        <is>
+          <t>NYY</t>
+        </is>
+      </c>
+      <c r="C118" s="1" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="D118" s="1" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E118" s="1" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="F118" s="1" t="inlineStr">
+        <is>
+          <t>48.9%</t>
+        </is>
+      </c>
+      <c r="G118" s="1" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="H118" s="1" t="inlineStr">
+        <is>
+          <t>+8.9%</t>
+        </is>
+      </c>
+      <c r="I118" s="1" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="J118" s="1" t="inlineStr">
+        <is>
+          <t>50.4%</t>
+        </is>
+      </c>
+      <c r="K118" s="1" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="L118" s="1" t="inlineStr">
+        <is>
+          <t>+9.7%</t>
+        </is>
+      </c>
+      <c r="M118" s="1" t="inlineStr"/>
+      <c r="N118" s="1" t="inlineStr"/>
+      <c r="O118" s="1" t="inlineStr"/>
+      <c r="P118" s="1" t="inlineStr"/>
+      <c r="Q118" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R118" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="S118" s="1" t="inlineStr">
+        <is>
+          <t>NYY</t>
+        </is>
+      </c>
+      <c r="T118" s="1" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="U118" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B119" s="1" t="inlineStr">
+        <is>
+          <t>NYY</t>
+        </is>
+      </c>
+      <c r="C119" s="1" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="D119" s="1" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E119" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F119" s="1" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="G119" s="1" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="H119" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I119" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="J119" s="1" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="K119" s="1" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="L119" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="M119" s="1" t="inlineStr"/>
+      <c r="N119" s="1" t="inlineStr"/>
+      <c r="O119" s="1" t="inlineStr"/>
+      <c r="P119" s="1" t="inlineStr"/>
+      <c r="Q119" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="R119" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="S119" s="1" t="inlineStr">
+        <is>
+          <t>NYY</t>
+        </is>
+      </c>
+      <c r="T119" s="1" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U119" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B120" s="1" t="inlineStr">
+        <is>
+          <t>KCR</t>
+        </is>
+      </c>
+      <c r="C120" s="1" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="D120" s="1" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E120" s="1" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="F120" s="1" t="inlineStr">
+        <is>
+          <t>55.1%</t>
+        </is>
+      </c>
+      <c r="G120" s="1" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H120" s="1" t="inlineStr">
+        <is>
+          <t>+5.1%</t>
+        </is>
+      </c>
+      <c r="I120" s="1" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="J120" s="1" t="inlineStr">
+        <is>
+          <t>56.8%</t>
+        </is>
+      </c>
+      <c r="K120" s="1" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="L120" s="1" t="inlineStr">
+        <is>
+          <t>+6.8%</t>
+        </is>
+      </c>
+      <c r="M120" s="1" t="inlineStr"/>
+      <c r="N120" s="1" t="inlineStr"/>
+      <c r="O120" s="1" t="inlineStr"/>
+      <c r="P120" s="1" t="inlineStr"/>
+      <c r="Q120" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R120" s="1" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="S120" s="1" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="T120" s="1" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="U120" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B121" s="1" t="inlineStr">
+        <is>
+          <t>KCR</t>
+        </is>
+      </c>
+      <c r="C121" s="1" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="D121" s="1" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E121" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F121" s="1" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="G121" s="1" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="H121" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I121" s="1" t="inlineStr">
+        <is>
+          <t>Under</t>
+        </is>
+      </c>
+      <c r="J121" s="1" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="K121" s="1" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="L121" s="1" t="inlineStr">
+        <is>
+          <t>-1.5 runs</t>
+        </is>
+      </c>
+      <c r="M121" s="1" t="inlineStr"/>
+      <c r="N121" s="1" t="inlineStr"/>
+      <c r="O121" s="1" t="inlineStr"/>
+      <c r="P121" s="1" t="inlineStr"/>
+      <c r="Q121" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R121" s="1" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="S121" s="1" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="T121" s="1" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U121" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B122" s="1" t="inlineStr">
+        <is>
+          <t>CHC</t>
+        </is>
+      </c>
+      <c r="C122" s="1" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="D122" s="1" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E122" s="1" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="F122" s="1" t="inlineStr">
+        <is>
+          <t>76.8%</t>
+        </is>
+      </c>
+      <c r="G122" s="1" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H122" s="1" t="inlineStr">
+        <is>
+          <t>+26.8%</t>
+        </is>
+      </c>
+      <c r="I122" s="1" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="J122" s="1" t="inlineStr">
+        <is>
+          <t>76.6%</t>
+        </is>
+      </c>
+      <c r="K122" s="1" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="L122" s="1" t="inlineStr">
+        <is>
+          <t>+26.6%</t>
+        </is>
+      </c>
+      <c r="M122" s="1" t="inlineStr"/>
+      <c r="N122" s="1" t="inlineStr"/>
+      <c r="O122" s="1" t="inlineStr"/>
+      <c r="P122" s="1" t="inlineStr"/>
+      <c r="Q122" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R122" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="S122" s="1" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="T122" s="1" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="U122" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B123" s="1" t="inlineStr">
+        <is>
+          <t>CHC</t>
+        </is>
+      </c>
+      <c r="C123" s="1" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="D123" s="1" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E123" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F123" s="1" t="inlineStr">
+        <is>
+          <t>7.9</t>
+        </is>
+      </c>
+      <c r="G123" s="1" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="H123" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I123" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="J123" s="1" t="inlineStr">
+        <is>
+          <t>7.9</t>
+        </is>
+      </c>
+      <c r="K123" s="1" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="L123" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="M123" s="1" t="inlineStr"/>
+      <c r="N123" s="1" t="inlineStr"/>
+      <c r="O123" s="1" t="inlineStr"/>
+      <c r="P123" s="1" t="inlineStr"/>
+      <c r="Q123" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R123" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="S123" s="1" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="T123" s="1" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U123" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B124" s="1" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="C124" s="1" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="D124" s="1" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E124" s="1" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="F124" s="1" t="inlineStr">
+        <is>
+          <t>67.5%</t>
+        </is>
+      </c>
+      <c r="G124" s="1" t="inlineStr">
+        <is>
+          <t>-116</t>
+        </is>
+      </c>
+      <c r="H124" s="1" t="inlineStr">
+        <is>
+          <t>+13.7%</t>
+        </is>
+      </c>
+      <c r="I124" s="1" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="J124" s="1" t="inlineStr">
+        <is>
+          <t>67.0%</t>
+        </is>
+      </c>
+      <c r="K124" s="1" t="inlineStr">
+        <is>
+          <t>-116</t>
+        </is>
+      </c>
+      <c r="L124" s="1" t="inlineStr">
+        <is>
+          <t>+13.2%</t>
+        </is>
+      </c>
+      <c r="M124" s="1" t="inlineStr"/>
+      <c r="N124" s="1" t="inlineStr"/>
+      <c r="O124" s="1" t="inlineStr"/>
+      <c r="P124" s="1" t="inlineStr"/>
+      <c r="Q124" s="1" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="R124" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="S124" s="1" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="T124" s="1" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="U124" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B125" s="1" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="C125" s="1" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="D125" s="1" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E125" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F125" s="1" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="G125" s="1" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="H125" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I125" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="J125" s="1" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="K125" s="1" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="L125" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="M125" s="1" t="inlineStr"/>
+      <c r="N125" s="1" t="inlineStr"/>
+      <c r="O125" s="1" t="inlineStr"/>
+      <c r="P125" s="1" t="inlineStr"/>
+      <c r="Q125" s="1" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="R125" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="S125" s="1" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="T125" s="1" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U125" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B126" s="1" t="inlineStr">
+        <is>
+          <t>SDP</t>
+        </is>
+      </c>
+      <c r="C126" s="1" t="inlineStr">
+        <is>
+          <t>LAD</t>
+        </is>
+      </c>
+      <c r="D126" s="1" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E126" s="1" t="inlineStr">
+        <is>
+          <t>LAD</t>
+        </is>
+      </c>
+      <c r="F126" s="1" t="inlineStr">
+        <is>
+          <t>75.5%</t>
+        </is>
+      </c>
+      <c r="G126" s="1" t="inlineStr">
+        <is>
+          <t>-175</t>
+        </is>
+      </c>
+      <c r="H126" s="1" t="inlineStr">
+        <is>
+          <t>+11.8%</t>
+        </is>
+      </c>
+      <c r="I126" s="1" t="inlineStr">
+        <is>
+          <t>LAD</t>
+        </is>
+      </c>
+      <c r="J126" s="1" t="inlineStr">
+        <is>
+          <t>75.9%</t>
+        </is>
+      </c>
+      <c r="K126" s="1" t="inlineStr">
+        <is>
+          <t>-186</t>
+        </is>
+      </c>
+      <c r="L126" s="1" t="inlineStr">
+        <is>
+          <t>+10.9%</t>
+        </is>
+      </c>
+      <c r="M126" s="1" t="inlineStr"/>
+      <c r="N126" s="1" t="inlineStr"/>
+      <c r="O126" s="1" t="inlineStr"/>
+      <c r="P126" s="1" t="inlineStr"/>
+      <c r="Q126" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R126" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="S126" s="1" t="inlineStr">
+        <is>
+          <t>LAD</t>
+        </is>
+      </c>
+      <c r="T126" s="1" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="U126" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B127" s="1" t="inlineStr">
+        <is>
+          <t>SDP</t>
+        </is>
+      </c>
+      <c r="C127" s="1" t="inlineStr">
+        <is>
+          <t>LAD</t>
+        </is>
+      </c>
+      <c r="D127" s="1" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E127" s="1" t="inlineStr">
+        <is>
+          <t>Under</t>
+        </is>
+      </c>
+      <c r="F127" s="1" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="G127" s="1" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="H127" s="1" t="inlineStr">
+        <is>
+          <t>-1.9 runs</t>
+        </is>
+      </c>
+      <c r="I127" s="1" t="inlineStr">
+        <is>
+          <t>Under</t>
+        </is>
+      </c>
+      <c r="J127" s="1" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="K127" s="1" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="L127" s="1" t="inlineStr">
+        <is>
+          <t>-1.9 runs</t>
+        </is>
+      </c>
+      <c r="M127" s="1" t="inlineStr"/>
+      <c r="N127" s="1" t="inlineStr"/>
+      <c r="O127" s="1" t="inlineStr"/>
+      <c r="P127" s="1" t="inlineStr"/>
+      <c r="Q127" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="R127" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="S127" s="1" t="inlineStr">
+        <is>
+          <t>LAD</t>
+        </is>
+      </c>
+      <c r="T127" s="1" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U127" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B128" s="1" t="inlineStr">
+        <is>
+          <t>LAA</t>
+        </is>
+      </c>
+      <c r="C128" s="1" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="D128" s="1" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E128" s="1" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="F128" s="1" t="inlineStr">
+        <is>
+          <t>77.9%</t>
+        </is>
+      </c>
+      <c r="G128" s="1" t="inlineStr">
+        <is>
+          <t>-125</t>
+        </is>
+      </c>
+      <c r="H128" s="1" t="inlineStr">
+        <is>
+          <t>+22.3%</t>
+        </is>
+      </c>
+      <c r="I128" s="1" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="J128" s="1" t="inlineStr">
+        <is>
+          <t>77.5%</t>
+        </is>
+      </c>
+      <c r="K128" s="1" t="inlineStr">
+        <is>
+          <t>-125</t>
+        </is>
+      </c>
+      <c r="L128" s="1" t="inlineStr">
+        <is>
+          <t>+22.0%</t>
+        </is>
+      </c>
+      <c r="M128" s="1" t="inlineStr"/>
+      <c r="N128" s="1" t="inlineStr"/>
+      <c r="O128" s="1" t="inlineStr"/>
+      <c r="P128" s="1" t="inlineStr"/>
+      <c r="Q128" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="R128" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="S128" s="1" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="T128" s="1" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="U128" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B129" s="1" t="inlineStr">
+        <is>
+          <t>LAA</t>
+        </is>
+      </c>
+      <c r="C129" s="1" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="D129" s="1" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="E129" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="F129" s="1" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="G129" s="1" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="H129" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="I129" s="1" t="inlineStr">
+        <is>
+          <t>No Bet</t>
+        </is>
+      </c>
+      <c r="J129" s="1" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="K129" s="1" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="L129" s="1" t="inlineStr">
+        <is>
+          <t>No Edge</t>
+        </is>
+      </c>
+      <c r="M129" s="1" t="inlineStr"/>
+      <c r="N129" s="1" t="inlineStr"/>
+      <c r="O129" s="1" t="inlineStr"/>
+      <c r="P129" s="1" t="inlineStr"/>
+      <c r="Q129" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="R129" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="S129" s="1" t="inlineStr">
+        <is>
+          <t>ATH</t>
+        </is>
+      </c>
+      <c r="T129" s="1" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U129" s="1" t="inlineStr">
+        <is>
+          <t>TEAM CHANGED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>